<commit_message>
organize and record smallBox data
</commit_message>
<xml_diff>
--- a/LA4/output/simpleBoxBlur/parallelConvolutionGraphs.xlsx
+++ b/LA4/output/simpleBoxBlur/parallelConvolutionGraphs.xlsx
@@ -5,16 +5,24 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crawfordd1\git\Labs\LA4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crawfordd1\git\Labs\LA4\output\simpleBoxBlur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{43F7A0C0-F89D-4F9B-991A-53EDDC0DEC06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74C1AA5-6F5A-48AB-B054-BD0C43DC3690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9FA3AC45-55BB-4246-9435-D247831757F4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9FA3AC45-55BB-4246-9435-D247831757F4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Box Kernel 31 px square" sheetId="1" r:id="rId1"/>
+    <sheet name="Box Kernel 11 px square" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'Box Kernel 31 px square'!$A$3</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Box Kernel 31 px square'!$A$4</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Box Kernel 31 px square'!$B$2:$H$2</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'Box Kernel 31 px square'!$B$3:$H$3</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'Box Kernel 31 px square'!$B$4:$H$4</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t xml:space="preserve">Number of Ranks: </t>
   </si>
@@ -57,6 +65,24 @@
   </si>
   <si>
     <t>Combined time (s):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full time: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bcast time: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calc time: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gather time: </t>
+  </si>
+  <si>
+    <t>Box kernel 11 px square</t>
+  </si>
+  <si>
+    <t>Combined time:</t>
   </si>
 </sst>
 </file>
@@ -206,7 +232,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$3</c:f>
+              <c:f>'Box Kernel 31 px square'!$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -241,7 +267,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$H$2</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$2:$H$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -271,7 +297,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$3:$H$3</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$3:$H$3</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -311,7 +337,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$4</c:f>
+              <c:f>'Box Kernel 31 px square'!$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -346,7 +372,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$H$2</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$2:$H$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -376,7 +402,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$4:$H$4</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$4:$H$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -850,7 +876,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$5</c:f>
+              <c:f>'Box Kernel 31 px square'!$A$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -885,7 +911,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$H$2</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$2:$H$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -915,7 +941,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$5:$H$5</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$5:$H$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -955,7 +981,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$6</c:f>
+              <c:f>'Box Kernel 31 px square'!$A$6</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -990,7 +1016,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$H$2</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$2:$H$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1020,7 +1046,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$6:$H$6</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$6:$H$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1060,7 +1086,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$7</c:f>
+              <c:f>'Box Kernel 31 px square'!$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1095,7 +1121,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$H$2</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$2:$H$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1125,7 +1151,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$7:$H$7</c:f>
+              <c:f>'Box Kernel 31 px square'!$B$7:$H$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1157,6 +1183,1429 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-AB81-4DD7-9B59-DED853D61114}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="768423007"/>
+        <c:axId val="768420607"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="768423007"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Number</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> of Ranks</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="768420607"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="768420607"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t>Time (s)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="768423007"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13459623797025372"/>
+          <c:y val="0.79305103148751355"/>
+          <c:w val="0.74318153980752399"/>
+          <c:h val="0.14169534997050451"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Box</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Convolution 31px Full Time</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.11082669914879424"/>
+          <c:y val="0.12928974260515086"/>
+          <c:w val="0.82751487555768233"/>
+          <c:h val="0.61860290345627733"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Box Kernel 11 px square'!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Full time: </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$2:$I$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$3:$I$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>8.6215250000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.587612</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.2640440000000002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.6011709999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.2533750000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.9966010000000001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.6308819999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.5819799999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FAFD-4AFC-A0A7-1EC2CAAC7764}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Box Kernel 11 px square'!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Calc time: </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$2:$I$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$4:$I$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>8.204917</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.1030449999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.7350089999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.049633</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.6400060000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.365183</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.81868099999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.68195899999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-FAFD-4AFC-A0A7-1EC2CAAC7764}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="768423007"/>
+        <c:axId val="768420607"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="768423007"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Number</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> of Ranks</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="768420607"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="768420607"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t>Time (s)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="768423007"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.24972279017608992"/>
+          <c:y val="0.85963352585956787"/>
+          <c:w val="0.56538139763779538"/>
+          <c:h val="0.13975253093363332"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Box</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Convolution 11px Parallel Costs</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.13187270341207349"/>
+          <c:y val="0.17171296296296296"/>
+          <c:w val="0.80950131233595801"/>
+          <c:h val="0.50734580052493439"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Box Kernel 11 px square'!$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Bcast time: </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$2:$I$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$5:$I$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1.9999999999999999E-6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.9012E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.6548E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.8816999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.9308999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.8606000000000003E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.372915</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.454405</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F1FA-4BF9-B351-D03A06D32F10}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Box Kernel 11 px square'!$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Gather time: </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$2:$I$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$6:$I$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.17904300000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.19358</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.20153799999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.26644000000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.324457</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.341223</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.204985</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.20336399999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F1FA-4BF9-B351-D03A06D32F10}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Box Kernel 11 px square'!$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Combined time:</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$2:$I$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Box Kernel 11 px square'!$B$7:$I$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.17904500000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.242592</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.28808600000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.305257</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.37376599999999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.38982899999999998</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.57789999999999997</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.65776900000000005</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-F1FA-4BF9-B351-D03A06D32F10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1584,6 +3033,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2101,6 +3630,1038 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2673,6 +5234,87 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81973EE7-6541-428D-9DCA-92EA9298ABE7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{560E83A1-33F5-4095-B7BF-9E18A40475D3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>9526</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68B7DD77-B258-4B62-AB7E-836F3F13C800}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3190,4 +5832,205 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3E99DDF-7FE3-427B-9E6E-060B6CCF39E4}">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>10</v>
+      </c>
+      <c r="I2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>8.6215250000000001</v>
+      </c>
+      <c r="C3">
+        <v>4.587612</v>
+      </c>
+      <c r="D3">
+        <v>3.2640440000000002</v>
+      </c>
+      <c r="E3">
+        <v>2.6011709999999999</v>
+      </c>
+      <c r="F3">
+        <v>2.2533750000000001</v>
+      </c>
+      <c r="G3">
+        <v>1.9966010000000001</v>
+      </c>
+      <c r="H3">
+        <v>1.6308819999999999</v>
+      </c>
+      <c r="I3">
+        <v>1.5819799999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>8.204917</v>
+      </c>
+      <c r="C4">
+        <v>4.1030449999999998</v>
+      </c>
+      <c r="D4">
+        <v>2.7350089999999998</v>
+      </c>
+      <c r="E4">
+        <v>2.049633</v>
+      </c>
+      <c r="F4">
+        <v>1.6400060000000001</v>
+      </c>
+      <c r="G4">
+        <v>1.365183</v>
+      </c>
+      <c r="H4">
+        <v>0.81868099999999999</v>
+      </c>
+      <c r="I4">
+        <v>0.68195899999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>1.9999999999999999E-6</v>
+      </c>
+      <c r="C5">
+        <v>4.9012E-2</v>
+      </c>
+      <c r="D5">
+        <v>8.6548E-2</v>
+      </c>
+      <c r="E5">
+        <v>3.8816999999999997E-2</v>
+      </c>
+      <c r="F5">
+        <v>4.9308999999999999E-2</v>
+      </c>
+      <c r="G5">
+        <v>4.8606000000000003E-2</v>
+      </c>
+      <c r="H5">
+        <v>0.372915</v>
+      </c>
+      <c r="I5">
+        <v>0.454405</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0.17904300000000001</v>
+      </c>
+      <c r="C6">
+        <v>0.19358</v>
+      </c>
+      <c r="D6">
+        <v>0.20153799999999999</v>
+      </c>
+      <c r="E6">
+        <v>0.26644000000000001</v>
+      </c>
+      <c r="F6">
+        <v>0.324457</v>
+      </c>
+      <c r="G6">
+        <v>0.341223</v>
+      </c>
+      <c r="H6">
+        <v>0.204985</v>
+      </c>
+      <c r="I6">
+        <v>0.20336399999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <f>B5+B6</f>
+        <v>0.17904500000000001</v>
+      </c>
+      <c r="C7">
+        <f t="shared" ref="C7:I7" si="0">C5+C6</f>
+        <v>0.242592</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>0.28808600000000001</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0.305257</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>0.37376599999999999</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>0.38982899999999998</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>0.57789999999999997</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>0.65776900000000005</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>